<commit_message>
feat: task_list_kyungnam에 특수관계자 분析 활성화
- 기존 11번(특수관계자분析) 실행여부 N→Y, 분析대상 당기→전체 수정
- 특수관계자 파라미터 시트 추가 (거래처명/실행여부 컬럼)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/kyungnam/task_list_kyungnam.xlsx
+++ b/journal_analyzer/kyungnam/task_list_kyungnam.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,25 +16,37 @@
     <sheet name="심층분석" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="거래처분석" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="벤포드이탈" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="특수관계자" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,10 +66,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -71,7 +91,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -435,7 +455,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -534,121 +554,168 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>금액열</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>임계값</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>최대건수</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>접대비</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>임계값 3%p 이상 이탈 건 추출</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>복리후생비</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D3" t="n">
+        <v>200</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>임계값 3%p 이상 이탈 건 추출</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>판매촉진비</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>임계값 3%p 이상 이탈 건 추출</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>계정과목</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>금액열</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>임계값</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>최대건수</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>비고</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>접대비</t>
-        </is>
-      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D2" t="n">
-        <v>200</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>임계값 3%p 이상 이탈 건 추출</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>복리후생비</t>
-        </is>
-      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D3" t="n">
-        <v>200</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>임계값 3%p 이상 이탈 건 추출</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>판매촉진비</t>
-        </is>
-      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D4" t="n">
-        <v>200</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>임계값 3%p 이상 이탈 건 추출</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -664,7 +731,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="15.25" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -934,12 +1004,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>전체</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1225,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1301,7 +1371,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1403,7 +1473,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1604,7 +1674,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1720,7 +1790,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1766,7 +1836,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1907,7 +1977,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1952,7 +2022,6 @@
           <t>접대비</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>차변</t>
@@ -1980,7 +2049,6 @@
           <t>판매촉진비</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>차변</t>
@@ -2003,8 +2071,6 @@
           <t>특수관계자_매출</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>대변</t>

</xml_diff>

<commit_message>
fix: AI_INJECT/ANALYSIS_INJECT 헤더 오프셋 버그 수정 + kyungnam AI검토 매핑 추가
- data_injector.py: inject_analysis_result/inject_ai_result가 분석결과 파일의
  1~2행(회사명/분석기간)을 헤더로 잘못 읽던 문제 수정 (header=2 지정)
  kyungnam 실제 실행으로 재현·수정 확인 (수정 전: 6열 전부 깨짐 → 수정 후 정상)
- task_list_kyungnam.xlsx: 26번(AI계정별분석_실행) 메뉴 등록 + 파라미터 시트(보통예금) 추가
- Kyungnam_mapping_list_25년.xlsx: AI검토결과/AI검토_확인전표 → 신규 'AI검토' 시트
  주입 매핑 행 2개 추가 (AI_INJECT), 실제 data_injector.py 전체 실행으로 검증 완료

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/kyungnam/task_list_kyungnam.xlsx
+++ b/journal_analyzer/kyungnam/task_list_kyungnam.xlsx
@@ -22,6 +22,7 @@
     <sheet name="은행조회서 완전성" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="거래처분析" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="손익월별분析" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="AI계정별분석_실행" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -197,7 +198,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -262,6 +263,7 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -2585,13 +2587,55 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3234,6 +3278,33 @@
           <t>전체</t>
         </is>
       </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>AI계정별분석_실행</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>계정별 월별 추이 및 샘플을 Gemini로 분석실행(15번 메뉴와 관계없이 독립적으로 실행)</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>